<commit_message>
Update dusty-cnc wiring diagram
Update the wiring chart to match wiring diagram:
- W15/16 changed to spade terminals
</commit_message>
<xml_diff>
--- a/documentation/wiring-diagram/Dustie Wiring Chart.export.xlsx
+++ b/documentation/wiring-diagram/Dustie Wiring Chart.export.xlsx
@@ -1210,1641 +1210,1644 @@
     <t>TB2:4→</t>
   </si>
   <si>
+    <t>SPADE</t>
+  </si>
+  <si>
+    <t>→ J35:N</t>
+  </si>
+  <si>
+    <t>TB2:14→</t>
+  </si>
+  <si>
+    <t>14</t>
+  </si>
+  <si>
+    <t>→ TB3:1</t>
+  </si>
+  <si>
+    <t>K1:T1→</t>
+  </si>
+  <si>
+    <t>T1</t>
+  </si>
+  <si>
+    <t>→ TB3:11</t>
+  </si>
+  <si>
+    <t>K1:T2→</t>
+  </si>
+  <si>
+    <t>T2</t>
+  </si>
+  <si>
+    <t>→ PS5:L</t>
+  </si>
+  <si>
+    <t>TB3:10→</t>
+  </si>
+  <si>
+    <t>→ PS5:N</t>
+  </si>
+  <si>
+    <t>TB3:20→</t>
+  </si>
+  <si>
+    <t>→ PS6:L</t>
+  </si>
+  <si>
+    <t>TB3:8→</t>
+  </si>
+  <si>
+    <t>→ PS6:N</t>
+  </si>
+  <si>
+    <t>TB3:18→</t>
+  </si>
+  <si>
+    <t>→ PS4:L</t>
+  </si>
+  <si>
+    <t>TB3:6→</t>
+  </si>
+  <si>
+    <t>→ PS4:N</t>
+  </si>
+  <si>
+    <t>TB3:16→</t>
+  </si>
+  <si>
+    <t>→ J6:4</t>
+  </si>
+  <si>
+    <t>TB3:4→</t>
+  </si>
+  <si>
+    <t>→ J6:3</t>
+  </si>
+  <si>
+    <t>TB3:14→</t>
+  </si>
+  <si>
+    <t>→ VFD1:R</t>
+  </si>
+  <si>
+    <t>P6:4→</t>
+  </si>
+  <si>
+    <t>Field</t>
+  </si>
+  <si>
+    <t>R</t>
+  </si>
+  <si>
+    <t>→ VFD1:S</t>
+  </si>
+  <si>
+    <t>P6:3→</t>
+  </si>
+  <si>
+    <t>S</t>
+  </si>
+  <si>
+    <t>→ J36:L</t>
+  </si>
+  <si>
+    <t>P35:L→</t>
+  </si>
+  <si>
+    <t>→ J36:N</t>
+  </si>
+  <si>
+    <t>P35:N→</t>
+  </si>
+  <si>
+    <t>→ TB5:1</t>
+  </si>
+  <si>
+    <t>PS1:V+→</t>
+  </si>
+  <si>
+    <t>Estop/Power Mgmt</t>
+  </si>
+  <si>
+    <t>24V_LOGIC</t>
+  </si>
+  <si>
+    <t>V+</t>
+  </si>
+  <si>
+    <t>🟦 Blue</t>
+  </si>
+  <si>
+    <t>→ TB5:9</t>
+  </si>
+  <si>
+    <t>PS1:V-→</t>
+  </si>
+  <si>
+    <t>0V_LOGIC</t>
+  </si>
+  <si>
+    <t>V-</t>
+  </si>
+  <si>
+    <t>🟦⬜️ Blue/White</t>
+  </si>
+  <si>
+    <t>→ S1:21</t>
+  </si>
+  <si>
+    <t>TB5:8→</t>
+  </si>
+  <si>
+    <t>→ S1:13</t>
+  </si>
+  <si>
+    <t>TB5:6→</t>
+  </si>
+  <si>
+    <t>→ J7:7</t>
+  </si>
+  <si>
+    <t>TB5:4→</t>
+  </si>
+  <si>
+    <t>→ J7:3</t>
+  </si>
+  <si>
+    <t>TB5:2→</t>
+  </si>
+  <si>
+    <t>→ PL1:X1</t>
+  </si>
+  <si>
+    <t>TB5:18→</t>
+  </si>
+  <si>
+    <t>ESTOP_INDICATOR</t>
+  </si>
+  <si>
+    <t>X1</t>
+  </si>
+  <si>
+    <t>→ J7:6</t>
+  </si>
+  <si>
+    <t>TB5:16→</t>
+  </si>
+  <si>
+    <t>→ J7:2</t>
+  </si>
+  <si>
+    <t>TB5:14→</t>
+  </si>
+  <si>
+    <t>→ PL4:X2</t>
+  </si>
+  <si>
+    <t>TB5:12→</t>
+  </si>
+  <si>
+    <t>12</t>
+  </si>
+  <si>
+    <t>X2</t>
+  </si>
+  <si>
+    <t>→ A2</t>
+  </si>
+  <si>
+    <t>TB5:10→</t>
+  </si>
+  <si>
+    <t>A2</t>
+  </si>
+  <si>
+    <t>→ TB8:1</t>
+  </si>
+  <si>
+    <t>S1:22→</t>
+  </si>
+  <si>
+    <t>ESTOP_LOOP</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>→ J7:8</t>
+  </si>
+  <si>
+    <t>TB8:2→</t>
+  </si>
+  <si>
+    <t>→ PL1:X2</t>
+  </si>
+  <si>
+    <t>S1:14→</t>
+  </si>
+  <si>
+    <t>→ TB9:1</t>
+  </si>
+  <si>
+    <t>J7:5→</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>→ J7:4</t>
+  </si>
+  <si>
+    <t>TB9:2→</t>
+  </si>
+  <si>
+    <t>→ TB10:1</t>
+  </si>
+  <si>
+    <t>J7:1→</t>
+  </si>
+  <si>
+    <t>→ PB2:21</t>
+  </si>
+  <si>
+    <t>TB10:2→</t>
+  </si>
+  <si>
+    <t>→ TB6:1</t>
+  </si>
+  <si>
+    <t>PB2:22→</t>
+  </si>
+  <si>
+    <t>→ PB1:13</t>
+  </si>
+  <si>
+    <t>TB6:2→</t>
+  </si>
+  <si>
+    <t>→ K1:13</t>
+  </si>
+  <si>
+    <t>TB6:4→</t>
+  </si>
+  <si>
+    <t>→ TB7:1</t>
+  </si>
+  <si>
+    <t>PB1:14→</t>
+  </si>
+  <si>
+    <t>MACHINE_ENABLE</t>
+  </si>
+  <si>
+    <t>→ K1:14</t>
+  </si>
+  <si>
+    <t>TB7:4→</t>
+  </si>
+  <si>
+    <t>→ K1:A1</t>
+  </si>
+  <si>
+    <t>TB7:6→</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>→ PL4:X1</t>
+  </si>
+  <si>
+    <t>TB7:2→</t>
+  </si>
+  <si>
+    <t>→ P12:8</t>
+  </si>
+  <si>
+    <t>P7:8→</t>
+  </si>
+  <si>
+    <t>→ P12:7</t>
+  </si>
+  <si>
+    <t>P7:7→</t>
+  </si>
+  <si>
+    <t>→ P12:6</t>
+  </si>
+  <si>
+    <t>P7:6→</t>
+  </si>
+  <si>
+    <t>→ P12:5</t>
+  </si>
+  <si>
+    <t>P7:5→</t>
+  </si>
+  <si>
+    <t>→ S2:21</t>
+  </si>
+  <si>
+    <t>J12:8→</t>
+  </si>
+  <si>
+    <t>→ S2:13</t>
+  </si>
+  <si>
+    <t>J12:7→</t>
+  </si>
+  <si>
+    <t>7</t>
+  </si>
+  <si>
+    <t>→ J12:6</t>
+  </si>
+  <si>
+    <t>PL2:X2→</t>
+  </si>
+  <si>
+    <t>→ J12:5</t>
+  </si>
+  <si>
+    <t>S2:22→</t>
+  </si>
+  <si>
+    <t>→ PL2:X1</t>
+  </si>
+  <si>
+    <t>S2:14→</t>
+  </si>
+  <si>
+    <t>→ P12:4</t>
+  </si>
+  <si>
+    <t>P7:4→</t>
+  </si>
+  <si>
+    <t>→ P12:3</t>
+  </si>
+  <si>
+    <t>P7:3→</t>
+  </si>
+  <si>
+    <t>→ P12:2</t>
+  </si>
+  <si>
+    <t>P7:2→</t>
+  </si>
+  <si>
+    <t>→ P12:1</t>
+  </si>
+  <si>
+    <t>P7:1→</t>
+  </si>
+  <si>
+    <t>→ J13:4</t>
+  </si>
+  <si>
+    <t>P12:4→</t>
+  </si>
+  <si>
+    <t>→ J13:3</t>
+  </si>
+  <si>
+    <t>P12:3→</t>
+  </si>
+  <si>
+    <t>→ J13:2</t>
+  </si>
+  <si>
+    <t>P12:2→</t>
+  </si>
+  <si>
+    <t>→ J13:1</t>
+  </si>
+  <si>
+    <t>P12:1→</t>
+  </si>
+  <si>
+    <t>→ P17:4</t>
+  </si>
+  <si>
+    <t>P13:4→</t>
+  </si>
+  <si>
+    <t>Flex optional</t>
+  </si>
+  <si>
+    <t>→ P17:3</t>
+  </si>
+  <si>
+    <t>P13:3→</t>
+  </si>
+  <si>
+    <t>→ P17:2</t>
+  </si>
+  <si>
+    <t>P13:2→</t>
+  </si>
+  <si>
+    <t>→ P17:1</t>
+  </si>
+  <si>
+    <t>P13:1→</t>
+  </si>
+  <si>
+    <t>→ S3:21</t>
+  </si>
+  <si>
+    <t>J17:4→</t>
+  </si>
+  <si>
+    <t>→ S3:13</t>
+  </si>
+  <si>
+    <t>J17:3→</t>
+  </si>
+  <si>
+    <t>→ J17:2</t>
+  </si>
+  <si>
+    <t>PL3:X2→</t>
+  </si>
+  <si>
+    <t>→ J17:1</t>
+  </si>
+  <si>
+    <t>S3:22→</t>
+  </si>
+  <si>
+    <t>→ PL3:X1</t>
+  </si>
+  <si>
+    <t>S3:14→</t>
+  </si>
+  <si>
+    <t>→ TB11:1</t>
+  </si>
+  <si>
+    <t>PS4:V+1→</t>
+  </si>
+  <si>
+    <t>24V Power</t>
+  </si>
+  <si>
+    <t>V+1</t>
+  </si>
+  <si>
+    <t>→ TB11:13</t>
+  </si>
+  <si>
+    <t>PS4:V-1→</t>
+  </si>
+  <si>
+    <t>V-1</t>
+  </si>
+  <si>
+    <t>→ MESA:TB3:22</t>
+  </si>
+  <si>
+    <t>TB11:2→</t>
+  </si>
+  <si>
+    <t>→ MESA:TB3:24</t>
+  </si>
+  <si>
+    <t>TB11:14→</t>
+  </si>
+  <si>
+    <t>→ MESA:TB1:5</t>
+  </si>
+  <si>
+    <t>TB11:4→</t>
+  </si>
+  <si>
+    <t>→ MESA:TB1:8</t>
+  </si>
+  <si>
+    <t>TB11:16→</t>
+  </si>
+  <si>
+    <t>→ FANS1:1</t>
+  </si>
+  <si>
+    <t>TB11:6→</t>
+  </si>
+  <si>
+    <t>FAN_PWR</t>
+  </si>
+  <si>
+    <t>FANS1</t>
+  </si>
+  <si>
+    <t>→ FANS1:2</t>
+  </si>
+  <si>
+    <t>TB11:18→</t>
+  </si>
+  <si>
+    <t>→ J2:1</t>
+  </si>
+  <si>
+    <t>TB11:8→</t>
+  </si>
+  <si>
+    <t>→ J2:2</t>
+  </si>
+  <si>
+    <t>TB11:20→</t>
+  </si>
+  <si>
+    <t>→ TI1:V+</t>
+  </si>
+  <si>
+    <t>TB11:10→</t>
+  </si>
+  <si>
+    <t>→ TI1:V-</t>
+  </si>
+  <si>
+    <t>TB11:22→</t>
+  </si>
+  <si>
+    <t>→ J4:2</t>
+  </si>
+  <si>
+    <t>MESA:TB6:17→</t>
+  </si>
+  <si>
+    <t>17</t>
+  </si>
+  <si>
+    <t>→ J4:1</t>
+  </si>
+  <si>
+    <t>TB11:24→</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>→ TI1:SIG</t>
+  </si>
+  <si>
+    <t>MESA:TB6:1→</t>
+  </si>
+  <si>
+    <t>TI1_VSENSE</t>
+  </si>
+  <si>
+    <t>SIG</t>
+  </si>
+  <si>
+    <t>→ P10:2</t>
+  </si>
+  <si>
+    <t>P2:2→</t>
+  </si>
+  <si>
+    <t>→ P10:1</t>
+  </si>
+  <si>
+    <t>P2:1→</t>
+  </si>
+  <si>
+    <t>→ TB51:1</t>
+  </si>
+  <si>
+    <t>J10:2→</t>
+  </si>
+  <si>
+    <t>→ TB52:1</t>
+  </si>
+  <si>
+    <t>J10:1→</t>
+  </si>
+  <si>
+    <t>→ J21:1</t>
+  </si>
+  <si>
+    <t>TB51:2→</t>
+  </si>
+  <si>
+    <t>→ J21:2</t>
+  </si>
+  <si>
+    <t>TB52:2→</t>
+  </si>
+  <si>
+    <t>→ LS1</t>
+  </si>
+  <si>
+    <t>TB51:3→</t>
+  </si>
+  <si>
+    <t>LIMIT_PWR</t>
+  </si>
+  <si>
+    <t>TB52:3→</t>
+  </si>
+  <si>
+    <t>LIMIT_GND</t>
+  </si>
+  <si>
+    <t>→ LS2</t>
+  </si>
+  <si>
+    <t>TB51:4→</t>
+  </si>
+  <si>
+    <t>TB52:4→</t>
+  </si>
+  <si>
+    <t>→ HS1</t>
+  </si>
+  <si>
+    <t>TB51:5→</t>
+  </si>
+  <si>
+    <t>TB52:5→</t>
+  </si>
+  <si>
+    <t>→ HS2</t>
+  </si>
+  <si>
+    <t>TB51:6→</t>
+  </si>
+  <si>
+    <t>TB52:6→</t>
+  </si>
+  <si>
+    <t>→ TP1</t>
+  </si>
+  <si>
+    <t>TB51:7→</t>
+  </si>
+  <si>
+    <t>PROBE_PWR</t>
+  </si>
+  <si>
+    <t>→ P20:2</t>
+  </si>
+  <si>
+    <t>P21:2→</t>
+  </si>
+  <si>
+    <t>→ P20:1</t>
+  </si>
+  <si>
+    <t>P21:1→</t>
+  </si>
+  <si>
+    <t>→ TB53:1</t>
+  </si>
+  <si>
+    <t>J20:2→</t>
+  </si>
+  <si>
+    <t>→ TB54:1</t>
+  </si>
+  <si>
+    <t>J20:1→</t>
+  </si>
+  <si>
+    <t>→ J25:1</t>
+  </si>
+  <si>
+    <t>TB53:2→</t>
+  </si>
+  <si>
+    <t>→ J25:2</t>
+  </si>
+  <si>
+    <t>TB54:2→</t>
+  </si>
+  <si>
+    <t>→ LS3</t>
+  </si>
+  <si>
+    <t>TB53:3→</t>
+  </si>
+  <si>
+    <t>TB54:3→</t>
+  </si>
+  <si>
+    <t>→ LS4</t>
+  </si>
+  <si>
+    <t>TB53:4→</t>
+  </si>
+  <si>
+    <t>TB54:4→</t>
+  </si>
+  <si>
+    <t>→ HS3</t>
+  </si>
+  <si>
+    <t>TB53:5→</t>
+  </si>
+  <si>
+    <t>TB54:5→</t>
+  </si>
+  <si>
+    <t>→ P29:2</t>
+  </si>
+  <si>
+    <t>P25:2→</t>
+  </si>
+  <si>
+    <t>→ P29:1</t>
+  </si>
+  <si>
+    <t>P25:1→</t>
+  </si>
+  <si>
+    <t>→ TB57:1</t>
+  </si>
+  <si>
+    <t>J29:2→</t>
+  </si>
+  <si>
+    <t>→ TB58:1</t>
+  </si>
+  <si>
+    <t>J29:1→</t>
+  </si>
+  <si>
+    <t>→ LS5</t>
+  </si>
+  <si>
+    <t>TB57:2→</t>
+  </si>
+  <si>
+    <t>TB58:2→</t>
+  </si>
+  <si>
+    <t>→ LS6</t>
+  </si>
+  <si>
+    <t>TB57:3→</t>
+  </si>
+  <si>
+    <t>TB58:3→</t>
+  </si>
+  <si>
+    <t>→ HS4</t>
+  </si>
+  <si>
+    <t>TB57:4→</t>
+  </si>
+  <si>
+    <t>TB58:4→</t>
+  </si>
+  <si>
+    <t>→ K2</t>
+  </si>
+  <si>
+    <t>P4:1→</t>
+  </si>
+  <si>
+    <t>Need suitable relay</t>
+  </si>
+  <si>
+    <t>P4:2→</t>
+  </si>
+  <si>
+    <t>→ J8:2</t>
+  </si>
+  <si>
+    <t>PS5:V+1→</t>
+  </si>
+  <si>
+    <t>48V Power</t>
+  </si>
+  <si>
+    <t>48V_LOGIC</t>
+  </si>
+  <si>
+    <t>🟧 Orange</t>
+  </si>
+  <si>
+    <t>→ J8:1</t>
+  </si>
+  <si>
+    <t>PS5:V-1→</t>
+  </si>
+  <si>
+    <t>🟫 Brown</t>
+  </si>
+  <si>
+    <t>→ J8:4</t>
+  </si>
+  <si>
+    <t>PS6:V+1→</t>
+  </si>
+  <si>
+    <t>→ J8:3</t>
+  </si>
+  <si>
+    <t>PS6:V-1→</t>
+  </si>
+  <si>
+    <t>→ SD2:DC+</t>
+  </si>
+  <si>
+    <t>PS6:V+2→</t>
+  </si>
+  <si>
+    <t>V+2</t>
+  </si>
+  <si>
+    <t>DC+</t>
+  </si>
+  <si>
+    <t>→ SD2:DC-</t>
+  </si>
+  <si>
+    <t>PS6:V-2→</t>
+  </si>
+  <si>
+    <t>V-2</t>
+  </si>
+  <si>
+    <t>DC-</t>
+  </si>
+  <si>
+    <t>PS6:V+3→</t>
+  </si>
+  <si>
+    <t>V+3</t>
+  </si>
+  <si>
+    <t>PS6:V-3→</t>
+  </si>
+  <si>
+    <t>V-3</t>
+  </si>
+  <si>
+    <t>→ P18:2</t>
+  </si>
+  <si>
+    <t>P8:2→</t>
+  </si>
+  <si>
+    <t>→ P18:1</t>
+  </si>
+  <si>
+    <t>P8:1→</t>
+  </si>
+  <si>
+    <t>→ P18:4</t>
+  </si>
+  <si>
+    <t>P8:4→</t>
+  </si>
+  <si>
+    <t>→ P18:3</t>
+  </si>
+  <si>
+    <t>P8:3→</t>
+  </si>
+  <si>
+    <t>→ J15:1</t>
+  </si>
+  <si>
+    <t>J18:2→</t>
+  </si>
+  <si>
+    <t>→ J15:2</t>
+  </si>
+  <si>
+    <t>J18:1→</t>
+  </si>
+  <si>
+    <t>→ J15:4</t>
+  </si>
+  <si>
+    <t>J18:4→</t>
+  </si>
+  <si>
+    <t>→ J15:3</t>
+  </si>
+  <si>
+    <t>J18:3→</t>
+  </si>
+  <si>
+    <t>→ P20:4</t>
+  </si>
+  <si>
+    <t>P15:2→</t>
+  </si>
+  <si>
+    <t>→ P20:3</t>
+  </si>
+  <si>
+    <t>P15:1→</t>
+  </si>
+  <si>
+    <t>→ P29:4</t>
+  </si>
+  <si>
+    <t>P15:4→</t>
+  </si>
+  <si>
+    <t>→ P29:3</t>
+  </si>
+  <si>
+    <t>P15:3→</t>
+  </si>
+  <si>
+    <t>→ TB55:1</t>
+  </si>
+  <si>
+    <t>J20:4→</t>
+  </si>
+  <si>
+    <t>→ TB56:1</t>
+  </si>
+  <si>
+    <t>J20:3→</t>
+  </si>
+  <si>
+    <t>→ IM1:VDC+</t>
+  </si>
+  <si>
+    <t>TB55:2→</t>
+  </si>
+  <si>
+    <t>STEP_IO_PWR</t>
+  </si>
+  <si>
+    <t>VDC+</t>
+  </si>
+  <si>
+    <t>→ IM1:GND</t>
+  </si>
+  <si>
+    <t>TB56:2→</t>
+  </si>
+  <si>
+    <t>STEP_IO_GND</t>
+  </si>
+  <si>
+    <t>GND</t>
+  </si>
+  <si>
+    <t>→ IM2:VDC+</t>
+  </si>
+  <si>
+    <t>TB55:3→</t>
+  </si>
+  <si>
+    <t>→ IM2:GND</t>
+  </si>
+  <si>
+    <t>TB56:4→</t>
+  </si>
+  <si>
+    <t>→ IM3:VDC+</t>
+  </si>
+  <si>
+    <t>J29:4→</t>
+  </si>
+  <si>
+    <t>→ IM3:GND</t>
+  </si>
+  <si>
+    <t>J29:3→</t>
+  </si>
+  <si>
+    <t>→ J5:2</t>
+  </si>
+  <si>
+    <t>MESA:TB3:18→</t>
+  </si>
+  <si>
+    <t>Control Signals</t>
+  </si>
+  <si>
+    <t>SPINDLE_RS+</t>
+  </si>
+  <si>
+    <t>🧵 Aqua</t>
+  </si>
+  <si>
+    <t>→ J5:1</t>
+  </si>
+  <si>
+    <t>MESA:TB3:16→</t>
+  </si>
+  <si>
+    <t>SPINDLE_RS-</t>
+  </si>
+  <si>
+    <t>🩵 Teal</t>
+  </si>
+  <si>
+    <t>→ J1:1</t>
+  </si>
+  <si>
+    <t>MESA:TB2:2→</t>
+  </si>
+  <si>
+    <t>Y1_STEP-</t>
+  </si>
+  <si>
+    <t>→ J1:2</t>
+  </si>
+  <si>
+    <t>MESA:TB2:3→</t>
+  </si>
+  <si>
+    <t>Y1_STEP+</t>
+  </si>
+  <si>
+    <t>→ J1:3</t>
+  </si>
+  <si>
+    <t>MESA:TB2:4→</t>
+  </si>
+  <si>
+    <t>Y1_DIR-</t>
+  </si>
+  <si>
+    <t>🟩⬜️ Green/White</t>
+  </si>
+  <si>
+    <t>→ J1:4</t>
+  </si>
+  <si>
+    <t>MESA:TB2:5→</t>
+  </si>
+  <si>
+    <t>Y1_DIR+</t>
+  </si>
+  <si>
+    <t>🟩 Green</t>
+  </si>
+  <si>
+    <t>→ J1:5</t>
+  </si>
+  <si>
+    <t>MESA:TB2:8→</t>
+  </si>
+  <si>
+    <t>Y2_STEP-</t>
+  </si>
+  <si>
+    <t>→ J1:6</t>
+  </si>
+  <si>
+    <t>MESA:TB2:9→</t>
+  </si>
+  <si>
+    <t>Y2_STEP+</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>→ J1:7</t>
+  </si>
+  <si>
+    <t>MESA:TB2:10→</t>
+  </si>
+  <si>
+    <t>Y2_DIR-</t>
+  </si>
+  <si>
+    <t>→ J1:8</t>
+  </si>
+  <si>
+    <t>MESA:TB2:11→</t>
+  </si>
+  <si>
+    <t>Y2_DIR+</t>
+  </si>
+  <si>
+    <t>11</t>
+  </si>
+  <si>
+    <t>→ J1:9</t>
+  </si>
+  <si>
+    <t>MESA:TB2:14→</t>
+  </si>
+  <si>
+    <t>X_STEP-</t>
+  </si>
+  <si>
+    <t>→ J1:10</t>
+  </si>
+  <si>
+    <t>MESA:TB2:15→</t>
+  </si>
+  <si>
+    <t>X_STEP+</t>
+  </si>
+  <si>
+    <t>15</t>
+  </si>
+  <si>
+    <t>→ J1:11</t>
+  </si>
+  <si>
+    <t>MESA:TB2:16→</t>
+  </si>
+  <si>
+    <t>X_DIR-</t>
+  </si>
+  <si>
+    <t>→ J1:12</t>
+  </si>
+  <si>
+    <t>MESA:TB2:17→</t>
+  </si>
+  <si>
+    <t>X_DIR+</t>
+  </si>
+  <si>
+    <t>→ SD1:PUL-</t>
+  </si>
+  <si>
+    <t>MESA:TB2:20→</t>
+  </si>
+  <si>
+    <t>Z_STEP-</t>
+  </si>
+  <si>
+    <t>PUL-</t>
+  </si>
+  <si>
+    <t>→ SD1:PUL+</t>
+  </si>
+  <si>
+    <t>MESA:TB2:21→</t>
+  </si>
+  <si>
+    <t>Z_STEP+</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>PUL+</t>
+  </si>
+  <si>
+    <t>→ SD1:DIR-</t>
+  </si>
+  <si>
+    <t>MESA:TB2:22→</t>
+  </si>
+  <si>
+    <t>Z_DIR-</t>
+  </si>
+  <si>
+    <t>DIR-</t>
+  </si>
+  <si>
+    <t>→ SD1:DIR+</t>
+  </si>
+  <si>
+    <t>MESA:TB2:23→</t>
+  </si>
+  <si>
+    <t>Z_DIR+</t>
+  </si>
+  <si>
+    <t>23</t>
+  </si>
+  <si>
+    <t>DIR+</t>
+  </si>
+  <si>
+    <t>→ J3:8</t>
+  </si>
+  <si>
+    <t>SD1:A+→</t>
+  </si>
+  <si>
+    <t>Z_A+</t>
+  </si>
+  <si>
+    <t>A+</t>
+  </si>
+  <si>
+    <t>Double check colours/order</t>
+  </si>
+  <si>
+    <t>→ J3:7</t>
+  </si>
+  <si>
+    <t>SD1:A-→</t>
+  </si>
+  <si>
+    <t>Z_A-</t>
+  </si>
+  <si>
+    <t>A-</t>
+  </si>
+  <si>
+    <t>→ J3:6</t>
+  </si>
+  <si>
+    <t>SD1:B+→</t>
+  </si>
+  <si>
+    <t>Z_B+</t>
+  </si>
+  <si>
+    <t>B+</t>
+  </si>
+  <si>
+    <t>→ J3:5</t>
+  </si>
+  <si>
+    <t>SD1:B-→</t>
+  </si>
+  <si>
+    <t>Z_B-</t>
+  </si>
+  <si>
+    <t>B-</t>
+  </si>
+  <si>
+    <t>→ J3:4</t>
+  </si>
+  <si>
+    <t>SD2:A+→</t>
+  </si>
+  <si>
+    <t>DUST_A+</t>
+  </si>
+  <si>
+    <t>→ J3:3</t>
+  </si>
+  <si>
+    <t>SD2:A-→</t>
+  </si>
+  <si>
+    <t>DUST_A-</t>
+  </si>
+  <si>
+    <t>→ J3:2</t>
+  </si>
+  <si>
+    <t>SD2:B+→</t>
+  </si>
+  <si>
+    <t>DUST_B+</t>
+  </si>
+  <si>
+    <t>→ J3:1</t>
+  </si>
+  <si>
+    <t>SD2:B-→</t>
+  </si>
+  <si>
+    <t>DUST_B-</t>
+  </si>
+  <si>
+    <t>→ J1:13</t>
+  </si>
+  <si>
+    <t>MESA:TB6:5→</t>
+  </si>
+  <si>
+    <t>Y_MIN</t>
+  </si>
+  <si>
+    <t>🩶 Grey</t>
+  </si>
+  <si>
+    <t>→ J1:14</t>
+  </si>
+  <si>
+    <t>MESA:TB6:6→</t>
+  </si>
+  <si>
+    <t>Y_MAX</t>
+  </si>
+  <si>
+    <t>→ J1:15</t>
+  </si>
+  <si>
+    <t>MESA:TB6:7→</t>
+  </si>
+  <si>
+    <t>Y1_HOME</t>
+  </si>
+  <si>
+    <t>→ J1:16</t>
+  </si>
+  <si>
+    <t>MESA:TB6:8→</t>
+  </si>
+  <si>
+    <t>Y2_HOME</t>
+  </si>
+  <si>
+    <t>→ J1:17</t>
+  </si>
+  <si>
+    <t>MESA:TB6:9→</t>
+  </si>
+  <si>
+    <t>X_MIN</t>
+  </si>
+  <si>
+    <t>→ J1:18</t>
+  </si>
+  <si>
+    <t>MESA:TB6:10→</t>
+  </si>
+  <si>
+    <t>X_MAX</t>
+  </si>
+  <si>
+    <t>→ J1:19</t>
+  </si>
+  <si>
+    <t>MESA:TB6:11→</t>
+  </si>
+  <si>
+    <t>X_HOME</t>
+  </si>
+  <si>
+    <t>→ J1:20</t>
+  </si>
+  <si>
+    <t>MESA:TB6:12→</t>
+  </si>
+  <si>
+    <t>Z_MIN</t>
+  </si>
+  <si>
+    <t>→ J1:21</t>
+  </si>
+  <si>
+    <t>MESA:TB6:13→</t>
+  </si>
+  <si>
+    <t>Z_MAX</t>
+  </si>
+  <si>
+    <t>13</t>
+  </si>
+  <si>
+    <t>→ J1:22</t>
+  </si>
+  <si>
+    <t>MESA:TB6:14→</t>
+  </si>
+  <si>
+    <t>Z_HOME</t>
+  </si>
+  <si>
+    <t>→ J1:23</t>
+  </si>
+  <si>
+    <t>MESA:TB6:15→</t>
+  </si>
+  <si>
+    <t>PROBE_IN</t>
+  </si>
+  <si>
+    <t>⬜️ White</t>
+  </si>
+  <si>
+    <t>→ FANS1:PWM</t>
+  </si>
+  <si>
+    <t>MESA:TB6:18→</t>
+  </si>
+  <si>
+    <t>FAN_PWM</t>
+  </si>
+  <si>
+    <t>PWM</t>
+  </si>
+  <si>
+    <t>→ J39:USB1</t>
+  </si>
+  <si>
+    <t>CPU1:USB1→</t>
+  </si>
+  <si>
+    <t>USB_HID</t>
+  </si>
+  <si>
+    <t>USB1</t>
+  </si>
+  <si>
+    <t>➖ not used</t>
+  </si>
+  <si>
+    <t>→ J38:USB1</t>
+  </si>
+  <si>
+    <t>CPU1:USB2→</t>
+  </si>
+  <si>
+    <t>USB_USER</t>
+  </si>
+  <si>
+    <t>USB2</t>
+  </si>
+  <si>
+    <t>Extend to monitor zone</t>
+  </si>
+  <si>
+    <t>→ J37:HDMI</t>
+  </si>
+  <si>
+    <t>CPU1:DP→</t>
+  </si>
+  <si>
+    <t>MONITOR</t>
+  </si>
+  <si>
+    <t>DP</t>
+  </si>
+  <si>
+    <t>Add in dp/hdmi adapter</t>
+  </si>
+  <si>
+    <t>→ RF1:1</t>
+  </si>
+  <si>
+    <t>CPU1:RF→</t>
+  </si>
+  <si>
+    <t>WIFI_EXT</t>
+  </si>
+  <si>
+    <t>RF</t>
+  </si>
+  <si>
+    <t>→ MESA:ETH</t>
+  </si>
+  <si>
+    <t>CPU1:ETH→</t>
+  </si>
+  <si>
+    <t>ETH_MESA</t>
+  </si>
+  <si>
+    <t>ETH</t>
+  </si>
+  <si>
+    <t>→ P11:8</t>
+  </si>
+  <si>
+    <t>P3:8→</t>
+  </si>
+  <si>
+    <t>→ P11:7</t>
+  </si>
+  <si>
+    <t>P3:7→</t>
+  </si>
+  <si>
+    <t>→ P11:6</t>
+  </si>
+  <si>
+    <t>P3:6→</t>
+  </si>
+  <si>
+    <t>→ P11:5</t>
+  </si>
+  <si>
+    <t>P3:5→</t>
+  </si>
+  <si>
+    <t>→ J18:1</t>
+  </si>
+  <si>
+    <t>J11:8→</t>
+  </si>
+  <si>
+    <t>→ J18:2</t>
+  </si>
+  <si>
+    <t>J11:7→</t>
+  </si>
+  <si>
+    <t>→ J18:3</t>
+  </si>
+  <si>
+    <t>J11:6→</t>
+  </si>
+  <si>
+    <t>→ J18:4</t>
+  </si>
+  <si>
+    <t>J11:5→</t>
+  </si>
+  <si>
+    <t>→ P30:8</t>
+  </si>
+  <si>
+    <t>P16:8→</t>
+  </si>
+  <si>
+    <t>→ P30:7</t>
+  </si>
+  <si>
+    <t>P16:7→</t>
+  </si>
+  <si>
+    <t>→ P30:6</t>
+  </si>
+  <si>
+    <t>P16:6→</t>
+  </si>
+  <si>
+    <t>→ P30:5</t>
+  </si>
+  <si>
+    <t>P16:5→</t>
+  </si>
+  <si>
+    <t>→ P11:4</t>
+  </si>
+  <si>
+    <t>P3:4→</t>
+  </si>
+  <si>
+    <t>→ P11:3</t>
+  </si>
+  <si>
+    <t>P3:3→</t>
+  </si>
+  <si>
+    <t>→ P11:2</t>
+  </si>
+  <si>
+    <t>P3:2→</t>
+  </si>
+  <si>
+    <t>→ P11:1</t>
+  </si>
+  <si>
+    <t>P3:1→</t>
+  </si>
+  <si>
+    <t>→ J16:4</t>
+  </si>
+  <si>
+    <t>J11:4→</t>
+  </si>
+  <si>
+    <t>→ J16:3</t>
+  </si>
+  <si>
+    <t>J11:3→</t>
+  </si>
+  <si>
+    <t>→ J16:2</t>
+  </si>
+  <si>
+    <t>J11:2→</t>
+  </si>
+  <si>
+    <t>→ J16:1</t>
+  </si>
+  <si>
+    <t>J11:1→</t>
+  </si>
+  <si>
+    <t>→ SM1</t>
+  </si>
+  <si>
+    <t>J30:8→</t>
+  </si>
+  <si>
+    <t>J30:7→</t>
+  </si>
+  <si>
+    <t>J30:6→</t>
+  </si>
+  <si>
+    <t>J30:5→</t>
+  </si>
+  <si>
+    <t>→ M1:1</t>
+  </si>
+  <si>
+    <t>VFD1:U→</t>
+  </si>
+  <si>
+    <t>SPINDLE_U</t>
+  </si>
+  <si>
+    <t>U</t>
+  </si>
+  <si>
     <t>SOLDER</t>
   </si>
   <si>
-    <t>→ J35:N</t>
-  </si>
-  <si>
-    <t>TB2:14→</t>
-  </si>
-  <si>
-    <t>14</t>
-  </si>
-  <si>
-    <t>→ TB3:1</t>
-  </si>
-  <si>
-    <t>K1:T1→</t>
-  </si>
-  <si>
-    <t>T1</t>
-  </si>
-  <si>
-    <t>→ TB3:11</t>
-  </si>
-  <si>
-    <t>K1:T2→</t>
-  </si>
-  <si>
-    <t>T2</t>
-  </si>
-  <si>
-    <t>→ PS5:L</t>
-  </si>
-  <si>
-    <t>TB3:10→</t>
-  </si>
-  <si>
-    <t>→ PS5:N</t>
-  </si>
-  <si>
-    <t>TB3:20→</t>
-  </si>
-  <si>
-    <t>→ PS6:L</t>
-  </si>
-  <si>
-    <t>TB3:8→</t>
-  </si>
-  <si>
-    <t>→ PS6:N</t>
-  </si>
-  <si>
-    <t>TB3:18→</t>
-  </si>
-  <si>
-    <t>→ PS4:L</t>
-  </si>
-  <si>
-    <t>TB3:6→</t>
-  </si>
-  <si>
-    <t>→ PS4:N</t>
-  </si>
-  <si>
-    <t>TB3:16→</t>
-  </si>
-  <si>
-    <t>→ J6:4</t>
-  </si>
-  <si>
-    <t>TB3:4→</t>
-  </si>
-  <si>
-    <t>→ J6:3</t>
-  </si>
-  <si>
-    <t>TB3:14→</t>
-  </si>
-  <si>
-    <t>→ VFD1:R</t>
-  </si>
-  <si>
-    <t>P6:4→</t>
-  </si>
-  <si>
-    <t>Field</t>
-  </si>
-  <si>
-    <t>R</t>
-  </si>
-  <si>
-    <t>→ VFD1:S</t>
-  </si>
-  <si>
-    <t>P6:3→</t>
-  </si>
-  <si>
-    <t>S</t>
-  </si>
-  <si>
-    <t>→ J36:L</t>
-  </si>
-  <si>
-    <t>P35:L→</t>
-  </si>
-  <si>
-    <t>→ J36:N</t>
-  </si>
-  <si>
-    <t>P35:N→</t>
-  </si>
-  <si>
-    <t>→ TB5:1</t>
-  </si>
-  <si>
-    <t>PS1:V+→</t>
-  </si>
-  <si>
-    <t>Estop/Power Mgmt</t>
-  </si>
-  <si>
-    <t>24V_LOGIC</t>
-  </si>
-  <si>
-    <t>V+</t>
-  </si>
-  <si>
-    <t>🟦 Blue</t>
-  </si>
-  <si>
-    <t>→ TB5:9</t>
-  </si>
-  <si>
-    <t>PS1:V-→</t>
-  </si>
-  <si>
-    <t>0V_LOGIC</t>
-  </si>
-  <si>
-    <t>V-</t>
-  </si>
-  <si>
-    <t>🟦⬜️ Blue/White</t>
-  </si>
-  <si>
-    <t>→ S1:21</t>
-  </si>
-  <si>
-    <t>TB5:8→</t>
-  </si>
-  <si>
-    <t>→ S1:13</t>
-  </si>
-  <si>
-    <t>TB5:6→</t>
-  </si>
-  <si>
-    <t>→ J7:7</t>
-  </si>
-  <si>
-    <t>TB5:4→</t>
-  </si>
-  <si>
-    <t>→ J7:3</t>
-  </si>
-  <si>
-    <t>TB5:2→</t>
-  </si>
-  <si>
-    <t>→ PL1:X1</t>
-  </si>
-  <si>
-    <t>TB5:18→</t>
-  </si>
-  <si>
-    <t>ESTOP_INDICATOR</t>
-  </si>
-  <si>
-    <t>X1</t>
-  </si>
-  <si>
-    <t>→ J7:6</t>
-  </si>
-  <si>
-    <t>TB5:16→</t>
-  </si>
-  <si>
-    <t>→ J7:2</t>
-  </si>
-  <si>
-    <t>TB5:14→</t>
-  </si>
-  <si>
-    <t>→ PL4:X2</t>
-  </si>
-  <si>
-    <t>TB5:12→</t>
-  </si>
-  <si>
-    <t>12</t>
-  </si>
-  <si>
-    <t>X2</t>
-  </si>
-  <si>
-    <t>→ A2</t>
-  </si>
-  <si>
-    <t>TB5:10→</t>
-  </si>
-  <si>
-    <t>A2</t>
-  </si>
-  <si>
-    <t>→ TB8:1</t>
-  </si>
-  <si>
-    <t>S1:22→</t>
-  </si>
-  <si>
-    <t>ESTOP_LOOP</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>→ J7:8</t>
-  </si>
-  <si>
-    <t>TB8:2→</t>
-  </si>
-  <si>
-    <t>→ PL1:X2</t>
-  </si>
-  <si>
-    <t>S1:14→</t>
-  </si>
-  <si>
-    <t>→ TB9:1</t>
-  </si>
-  <si>
-    <t>J7:5→</t>
-  </si>
-  <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>→ J7:4</t>
-  </si>
-  <si>
-    <t>TB9:2→</t>
-  </si>
-  <si>
-    <t>→ TB10:1</t>
-  </si>
-  <si>
-    <t>J7:1→</t>
-  </si>
-  <si>
-    <t>→ PB2:21</t>
-  </si>
-  <si>
-    <t>TB10:2→</t>
-  </si>
-  <si>
-    <t>→ TB6:1</t>
-  </si>
-  <si>
-    <t>PB2:22→</t>
-  </si>
-  <si>
-    <t>→ PB1:13</t>
-  </si>
-  <si>
-    <t>TB6:2→</t>
-  </si>
-  <si>
-    <t>→ K1:13</t>
-  </si>
-  <si>
-    <t>TB6:4→</t>
-  </si>
-  <si>
-    <t>→ TB7:1</t>
-  </si>
-  <si>
-    <t>PB1:14→</t>
-  </si>
-  <si>
-    <t>MACHINE_ENABLE</t>
-  </si>
-  <si>
-    <t>→ K1:14</t>
-  </si>
-  <si>
-    <t>TB7:4→</t>
-  </si>
-  <si>
-    <t>→ K1:A1</t>
-  </si>
-  <si>
-    <t>TB7:6→</t>
-  </si>
-  <si>
-    <t>A1</t>
-  </si>
-  <si>
-    <t>→ PL4:X1</t>
-  </si>
-  <si>
-    <t>TB7:2→</t>
-  </si>
-  <si>
-    <t>→ P12:8</t>
-  </si>
-  <si>
-    <t>P7:8→</t>
-  </si>
-  <si>
-    <t>→ P12:7</t>
-  </si>
-  <si>
-    <t>P7:7→</t>
-  </si>
-  <si>
-    <t>→ P12:6</t>
-  </si>
-  <si>
-    <t>P7:6→</t>
-  </si>
-  <si>
-    <t>→ P12:5</t>
-  </si>
-  <si>
-    <t>P7:5→</t>
-  </si>
-  <si>
-    <t>→ S2:21</t>
-  </si>
-  <si>
-    <t>J12:8→</t>
-  </si>
-  <si>
-    <t>→ S2:13</t>
-  </si>
-  <si>
-    <t>J12:7→</t>
-  </si>
-  <si>
-    <t>7</t>
-  </si>
-  <si>
-    <t>→ J12:6</t>
-  </si>
-  <si>
-    <t>PL2:X2→</t>
-  </si>
-  <si>
-    <t>→ J12:5</t>
-  </si>
-  <si>
-    <t>S2:22→</t>
-  </si>
-  <si>
-    <t>→ PL2:X1</t>
-  </si>
-  <si>
-    <t>S2:14→</t>
-  </si>
-  <si>
-    <t>→ P12:4</t>
-  </si>
-  <si>
-    <t>P7:4→</t>
-  </si>
-  <si>
-    <t>→ P12:3</t>
-  </si>
-  <si>
-    <t>P7:3→</t>
-  </si>
-  <si>
-    <t>→ P12:2</t>
-  </si>
-  <si>
-    <t>P7:2→</t>
-  </si>
-  <si>
-    <t>→ P12:1</t>
-  </si>
-  <si>
-    <t>P7:1→</t>
-  </si>
-  <si>
-    <t>→ J13:4</t>
-  </si>
-  <si>
-    <t>P12:4→</t>
-  </si>
-  <si>
-    <t>→ J13:3</t>
-  </si>
-  <si>
-    <t>P12:3→</t>
-  </si>
-  <si>
-    <t>→ J13:2</t>
-  </si>
-  <si>
-    <t>P12:2→</t>
-  </si>
-  <si>
-    <t>→ J13:1</t>
-  </si>
-  <si>
-    <t>P12:1→</t>
-  </si>
-  <si>
-    <t>→ P17:4</t>
-  </si>
-  <si>
-    <t>P13:4→</t>
-  </si>
-  <si>
-    <t>Flex optional</t>
-  </si>
-  <si>
-    <t>→ P17:3</t>
-  </si>
-  <si>
-    <t>P13:3→</t>
-  </si>
-  <si>
-    <t>→ P17:2</t>
-  </si>
-  <si>
-    <t>P13:2→</t>
-  </si>
-  <si>
-    <t>→ P17:1</t>
-  </si>
-  <si>
-    <t>P13:1→</t>
-  </si>
-  <si>
-    <t>→ S3:21</t>
-  </si>
-  <si>
-    <t>J17:4→</t>
-  </si>
-  <si>
-    <t>→ S3:13</t>
-  </si>
-  <si>
-    <t>J17:3→</t>
-  </si>
-  <si>
-    <t>→ J17:2</t>
-  </si>
-  <si>
-    <t>PL3:X2→</t>
-  </si>
-  <si>
-    <t>→ J17:1</t>
-  </si>
-  <si>
-    <t>S3:22→</t>
-  </si>
-  <si>
-    <t>→ PL3:X1</t>
-  </si>
-  <si>
-    <t>S3:14→</t>
-  </si>
-  <si>
-    <t>→ TB11:1</t>
-  </si>
-  <si>
-    <t>PS4:V+1→</t>
-  </si>
-  <si>
-    <t>24V Power</t>
-  </si>
-  <si>
-    <t>V+1</t>
-  </si>
-  <si>
-    <t>→ TB11:13</t>
-  </si>
-  <si>
-    <t>PS4:V-1→</t>
-  </si>
-  <si>
-    <t>V-1</t>
-  </si>
-  <si>
-    <t>→ MESA:TB3:22</t>
-  </si>
-  <si>
-    <t>TB11:2→</t>
-  </si>
-  <si>
-    <t>→ MESA:TB3:24</t>
-  </si>
-  <si>
-    <t>TB11:14→</t>
-  </si>
-  <si>
-    <t>→ MESA:TB1:5</t>
-  </si>
-  <si>
-    <t>TB11:4→</t>
-  </si>
-  <si>
-    <t>→ MESA:TB1:8</t>
-  </si>
-  <si>
-    <t>TB11:16→</t>
-  </si>
-  <si>
-    <t>→ FANS1:1</t>
-  </si>
-  <si>
-    <t>TB11:6→</t>
-  </si>
-  <si>
-    <t>FAN_PWR</t>
-  </si>
-  <si>
-    <t>FANS1</t>
-  </si>
-  <si>
-    <t>→ FANS1:2</t>
-  </si>
-  <si>
-    <t>TB11:18→</t>
-  </si>
-  <si>
-    <t>→ J2:1</t>
-  </si>
-  <si>
-    <t>TB11:8→</t>
-  </si>
-  <si>
-    <t>→ J2:2</t>
-  </si>
-  <si>
-    <t>TB11:20→</t>
-  </si>
-  <si>
-    <t>→ TI1:V+</t>
-  </si>
-  <si>
-    <t>TB11:10→</t>
-  </si>
-  <si>
-    <t>→ TI1:V-</t>
-  </si>
-  <si>
-    <t>TB11:22→</t>
-  </si>
-  <si>
-    <t>→ J4:2</t>
-  </si>
-  <si>
-    <t>MESA:TB6:17→</t>
-  </si>
-  <si>
-    <t>17</t>
-  </si>
-  <si>
-    <t>→ J4:1</t>
-  </si>
-  <si>
-    <t>TB11:24→</t>
-  </si>
-  <si>
-    <t>24</t>
-  </si>
-  <si>
-    <t>→ TI1:SIG</t>
-  </si>
-  <si>
-    <t>MESA:TB6:1→</t>
-  </si>
-  <si>
-    <t>TI1_VSENSE</t>
-  </si>
-  <si>
-    <t>SIG</t>
-  </si>
-  <si>
-    <t>→ P10:2</t>
-  </si>
-  <si>
-    <t>P2:2→</t>
-  </si>
-  <si>
-    <t>→ P10:1</t>
-  </si>
-  <si>
-    <t>P2:1→</t>
-  </si>
-  <si>
-    <t>→ TB51:1</t>
-  </si>
-  <si>
-    <t>J10:2→</t>
-  </si>
-  <si>
-    <t>→ TB52:1</t>
-  </si>
-  <si>
-    <t>J10:1→</t>
-  </si>
-  <si>
-    <t>→ J21:1</t>
-  </si>
-  <si>
-    <t>TB51:2→</t>
-  </si>
-  <si>
-    <t>→ J21:2</t>
-  </si>
-  <si>
-    <t>TB52:2→</t>
-  </si>
-  <si>
-    <t>→ LS1</t>
-  </si>
-  <si>
-    <t>TB51:3→</t>
-  </si>
-  <si>
-    <t>LIMIT_PWR</t>
-  </si>
-  <si>
-    <t>TB52:3→</t>
-  </si>
-  <si>
-    <t>LIMIT_GND</t>
-  </si>
-  <si>
-    <t>→ LS2</t>
-  </si>
-  <si>
-    <t>TB51:4→</t>
-  </si>
-  <si>
-    <t>TB52:4→</t>
-  </si>
-  <si>
-    <t>→ HS1</t>
-  </si>
-  <si>
-    <t>TB51:5→</t>
-  </si>
-  <si>
-    <t>TB52:5→</t>
-  </si>
-  <si>
-    <t>→ HS2</t>
-  </si>
-  <si>
-    <t>TB51:6→</t>
-  </si>
-  <si>
-    <t>TB52:6→</t>
-  </si>
-  <si>
-    <t>→ TP1</t>
-  </si>
-  <si>
-    <t>TB51:7→</t>
-  </si>
-  <si>
-    <t>PROBE_PWR</t>
-  </si>
-  <si>
-    <t>→ P20:2</t>
-  </si>
-  <si>
-    <t>P21:2→</t>
-  </si>
-  <si>
-    <t>→ P20:1</t>
-  </si>
-  <si>
-    <t>P21:1→</t>
-  </si>
-  <si>
-    <t>→ TB53:1</t>
-  </si>
-  <si>
-    <t>J20:2→</t>
-  </si>
-  <si>
-    <t>→ TB54:1</t>
-  </si>
-  <si>
-    <t>J20:1→</t>
-  </si>
-  <si>
-    <t>→ J25:1</t>
-  </si>
-  <si>
-    <t>TB53:2→</t>
-  </si>
-  <si>
-    <t>→ J25:2</t>
-  </si>
-  <si>
-    <t>TB54:2→</t>
-  </si>
-  <si>
-    <t>→ LS3</t>
-  </si>
-  <si>
-    <t>TB53:3→</t>
-  </si>
-  <si>
-    <t>TB54:3→</t>
-  </si>
-  <si>
-    <t>→ LS4</t>
-  </si>
-  <si>
-    <t>TB53:4→</t>
-  </si>
-  <si>
-    <t>TB54:4→</t>
-  </si>
-  <si>
-    <t>→ HS3</t>
-  </si>
-  <si>
-    <t>TB53:5→</t>
-  </si>
-  <si>
-    <t>TB54:5→</t>
-  </si>
-  <si>
-    <t>→ P29:2</t>
-  </si>
-  <si>
-    <t>P25:2→</t>
-  </si>
-  <si>
-    <t>→ P29:1</t>
-  </si>
-  <si>
-    <t>P25:1→</t>
-  </si>
-  <si>
-    <t>→ TB57:1</t>
-  </si>
-  <si>
-    <t>J29:2→</t>
-  </si>
-  <si>
-    <t>→ TB58:1</t>
-  </si>
-  <si>
-    <t>J29:1→</t>
-  </si>
-  <si>
-    <t>→ LS5</t>
-  </si>
-  <si>
-    <t>TB57:2→</t>
-  </si>
-  <si>
-    <t>TB58:2→</t>
-  </si>
-  <si>
-    <t>→ LS6</t>
-  </si>
-  <si>
-    <t>TB57:3→</t>
-  </si>
-  <si>
-    <t>TB58:3→</t>
-  </si>
-  <si>
-    <t>→ HS4</t>
-  </si>
-  <si>
-    <t>TB57:4→</t>
-  </si>
-  <si>
-    <t>TB58:4→</t>
-  </si>
-  <si>
-    <t>→ K2</t>
-  </si>
-  <si>
-    <t>P4:1→</t>
-  </si>
-  <si>
-    <t>Need suitable relay</t>
-  </si>
-  <si>
-    <t>P4:2→</t>
-  </si>
-  <si>
-    <t>→ J8:2</t>
-  </si>
-  <si>
-    <t>PS5:V+1→</t>
-  </si>
-  <si>
-    <t>48V Power</t>
-  </si>
-  <si>
-    <t>48V_LOGIC</t>
-  </si>
-  <si>
-    <t>🟧 Orange</t>
-  </si>
-  <si>
-    <t>→ J8:1</t>
-  </si>
-  <si>
-    <t>PS5:V-1→</t>
-  </si>
-  <si>
-    <t>🟫 Brown</t>
-  </si>
-  <si>
-    <t>→ J8:4</t>
-  </si>
-  <si>
-    <t>PS6:V+1→</t>
-  </si>
-  <si>
-    <t>→ J8:3</t>
-  </si>
-  <si>
-    <t>PS6:V-1→</t>
-  </si>
-  <si>
-    <t>→ SD2:DC+</t>
-  </si>
-  <si>
-    <t>PS6:V+2→</t>
-  </si>
-  <si>
-    <t>V+2</t>
-  </si>
-  <si>
-    <t>DC+</t>
-  </si>
-  <si>
-    <t>→ SD2:DC-</t>
-  </si>
-  <si>
-    <t>PS6:V-2→</t>
-  </si>
-  <si>
-    <t>V-2</t>
-  </si>
-  <si>
-    <t>DC-</t>
-  </si>
-  <si>
-    <t>PS6:V+3→</t>
-  </si>
-  <si>
-    <t>V+3</t>
-  </si>
-  <si>
-    <t>PS6:V-3→</t>
-  </si>
-  <si>
-    <t>V-3</t>
-  </si>
-  <si>
-    <t>→ P18:2</t>
-  </si>
-  <si>
-    <t>P8:2→</t>
-  </si>
-  <si>
-    <t>→ P18:1</t>
-  </si>
-  <si>
-    <t>P8:1→</t>
-  </si>
-  <si>
-    <t>→ P18:4</t>
-  </si>
-  <si>
-    <t>P8:4→</t>
-  </si>
-  <si>
-    <t>→ P18:3</t>
-  </si>
-  <si>
-    <t>P8:3→</t>
-  </si>
-  <si>
-    <t>→ J15:1</t>
-  </si>
-  <si>
-    <t>J18:2→</t>
-  </si>
-  <si>
-    <t>→ J15:2</t>
-  </si>
-  <si>
-    <t>J18:1→</t>
-  </si>
-  <si>
-    <t>→ J15:4</t>
-  </si>
-  <si>
-    <t>J18:4→</t>
-  </si>
-  <si>
-    <t>→ J15:3</t>
-  </si>
-  <si>
-    <t>J18:3→</t>
-  </si>
-  <si>
-    <t>→ P20:4</t>
-  </si>
-  <si>
-    <t>P15:2→</t>
-  </si>
-  <si>
-    <t>→ P20:3</t>
-  </si>
-  <si>
-    <t>P15:1→</t>
-  </si>
-  <si>
-    <t>→ P29:4</t>
-  </si>
-  <si>
-    <t>P15:4→</t>
-  </si>
-  <si>
-    <t>→ P29:3</t>
-  </si>
-  <si>
-    <t>P15:3→</t>
-  </si>
-  <si>
-    <t>→ TB55:1</t>
-  </si>
-  <si>
-    <t>J20:4→</t>
-  </si>
-  <si>
-    <t>→ TB56:1</t>
-  </si>
-  <si>
-    <t>J20:3→</t>
-  </si>
-  <si>
-    <t>→ IM1:VDC+</t>
-  </si>
-  <si>
-    <t>TB55:2→</t>
-  </si>
-  <si>
-    <t>STEP_IO_PWR</t>
-  </si>
-  <si>
-    <t>VDC+</t>
-  </si>
-  <si>
-    <t>→ IM1:GND</t>
-  </si>
-  <si>
-    <t>TB56:2→</t>
-  </si>
-  <si>
-    <t>STEP_IO_GND</t>
-  </si>
-  <si>
-    <t>GND</t>
-  </si>
-  <si>
-    <t>→ IM2:VDC+</t>
-  </si>
-  <si>
-    <t>TB55:3→</t>
-  </si>
-  <si>
-    <t>→ IM2:GND</t>
-  </si>
-  <si>
-    <t>TB56:4→</t>
-  </si>
-  <si>
-    <t>→ IM3:VDC+</t>
-  </si>
-  <si>
-    <t>J29:4→</t>
-  </si>
-  <si>
-    <t>→ IM3:GND</t>
-  </si>
-  <si>
-    <t>J29:3→</t>
-  </si>
-  <si>
-    <t>→ J5:2</t>
-  </si>
-  <si>
-    <t>MESA:TB3:18→</t>
-  </si>
-  <si>
-    <t>Control Signals</t>
-  </si>
-  <si>
-    <t>SPINDLE_RS+</t>
-  </si>
-  <si>
-    <t>🧵 Aqua</t>
-  </si>
-  <si>
-    <t>→ J5:1</t>
-  </si>
-  <si>
-    <t>MESA:TB3:16→</t>
-  </si>
-  <si>
-    <t>SPINDLE_RS-</t>
-  </si>
-  <si>
-    <t>🩵 Teal</t>
-  </si>
-  <si>
-    <t>→ J1:1</t>
-  </si>
-  <si>
-    <t>MESA:TB2:2→</t>
-  </si>
-  <si>
-    <t>Y1_STEP-</t>
-  </si>
-  <si>
-    <t>→ J1:2</t>
-  </si>
-  <si>
-    <t>MESA:TB2:3→</t>
-  </si>
-  <si>
-    <t>Y1_STEP+</t>
-  </si>
-  <si>
-    <t>→ J1:3</t>
-  </si>
-  <si>
-    <t>MESA:TB2:4→</t>
-  </si>
-  <si>
-    <t>Y1_DIR-</t>
-  </si>
-  <si>
-    <t>🟩⬜️ Green/White</t>
-  </si>
-  <si>
-    <t>→ J1:4</t>
-  </si>
-  <si>
-    <t>MESA:TB2:5→</t>
-  </si>
-  <si>
-    <t>Y1_DIR+</t>
-  </si>
-  <si>
-    <t>🟩 Green</t>
-  </si>
-  <si>
-    <t>→ J1:5</t>
-  </si>
-  <si>
-    <t>MESA:TB2:8→</t>
-  </si>
-  <si>
-    <t>Y2_STEP-</t>
-  </si>
-  <si>
-    <t>→ J1:6</t>
-  </si>
-  <si>
-    <t>MESA:TB2:9→</t>
-  </si>
-  <si>
-    <t>Y2_STEP+</t>
-  </si>
-  <si>
-    <t>9</t>
-  </si>
-  <si>
-    <t>→ J1:7</t>
-  </si>
-  <si>
-    <t>MESA:TB2:10→</t>
-  </si>
-  <si>
-    <t>Y2_DIR-</t>
-  </si>
-  <si>
-    <t>→ J1:8</t>
-  </si>
-  <si>
-    <t>MESA:TB2:11→</t>
-  </si>
-  <si>
-    <t>Y2_DIR+</t>
-  </si>
-  <si>
-    <t>11</t>
-  </si>
-  <si>
-    <t>→ J1:9</t>
-  </si>
-  <si>
-    <t>MESA:TB2:14→</t>
-  </si>
-  <si>
-    <t>X_STEP-</t>
-  </si>
-  <si>
-    <t>→ J1:10</t>
-  </si>
-  <si>
-    <t>MESA:TB2:15→</t>
-  </si>
-  <si>
-    <t>X_STEP+</t>
-  </si>
-  <si>
-    <t>15</t>
-  </si>
-  <si>
-    <t>→ J1:11</t>
-  </si>
-  <si>
-    <t>MESA:TB2:16→</t>
-  </si>
-  <si>
-    <t>X_DIR-</t>
-  </si>
-  <si>
-    <t>→ J1:12</t>
-  </si>
-  <si>
-    <t>MESA:TB2:17→</t>
-  </si>
-  <si>
-    <t>X_DIR+</t>
-  </si>
-  <si>
-    <t>→ SD1:PUL-</t>
-  </si>
-  <si>
-    <t>MESA:TB2:20→</t>
-  </si>
-  <si>
-    <t>Z_STEP-</t>
-  </si>
-  <si>
-    <t>PUL-</t>
-  </si>
-  <si>
-    <t>→ SD1:PUL+</t>
-  </si>
-  <si>
-    <t>MESA:TB2:21→</t>
-  </si>
-  <si>
-    <t>Z_STEP+</t>
-  </si>
-  <si>
-    <t>21</t>
-  </si>
-  <si>
-    <t>PUL+</t>
-  </si>
-  <si>
-    <t>→ SD1:DIR-</t>
-  </si>
-  <si>
-    <t>MESA:TB2:22→</t>
-  </si>
-  <si>
-    <t>Z_DIR-</t>
-  </si>
-  <si>
-    <t>DIR-</t>
-  </si>
-  <si>
-    <t>→ SD1:DIR+</t>
-  </si>
-  <si>
-    <t>MESA:TB2:23→</t>
-  </si>
-  <si>
-    <t>Z_DIR+</t>
-  </si>
-  <si>
-    <t>23</t>
-  </si>
-  <si>
-    <t>DIR+</t>
-  </si>
-  <si>
-    <t>→ J3:8</t>
-  </si>
-  <si>
-    <t>SD1:A+→</t>
-  </si>
-  <si>
-    <t>Z_A+</t>
-  </si>
-  <si>
-    <t>A+</t>
-  </si>
-  <si>
-    <t>Double check colours/order</t>
-  </si>
-  <si>
-    <t>→ J3:7</t>
-  </si>
-  <si>
-    <t>SD1:A-→</t>
-  </si>
-  <si>
-    <t>Z_A-</t>
-  </si>
-  <si>
-    <t>A-</t>
-  </si>
-  <si>
-    <t>→ J3:6</t>
-  </si>
-  <si>
-    <t>SD1:B+→</t>
-  </si>
-  <si>
-    <t>Z_B+</t>
-  </si>
-  <si>
-    <t>B+</t>
-  </si>
-  <si>
-    <t>→ J3:5</t>
-  </si>
-  <si>
-    <t>SD1:B-→</t>
-  </si>
-  <si>
-    <t>Z_B-</t>
-  </si>
-  <si>
-    <t>B-</t>
-  </si>
-  <si>
-    <t>→ J3:4</t>
-  </si>
-  <si>
-    <t>SD2:A+→</t>
-  </si>
-  <si>
-    <t>DUST_A+</t>
-  </si>
-  <si>
-    <t>→ J3:3</t>
-  </si>
-  <si>
-    <t>SD2:A-→</t>
-  </si>
-  <si>
-    <t>DUST_A-</t>
-  </si>
-  <si>
-    <t>→ J3:2</t>
-  </si>
-  <si>
-    <t>SD2:B+→</t>
-  </si>
-  <si>
-    <t>DUST_B+</t>
-  </si>
-  <si>
-    <t>→ J3:1</t>
-  </si>
-  <si>
-    <t>SD2:B-→</t>
-  </si>
-  <si>
-    <t>DUST_B-</t>
-  </si>
-  <si>
-    <t>→ J1:13</t>
-  </si>
-  <si>
-    <t>MESA:TB6:5→</t>
-  </si>
-  <si>
-    <t>Y_MIN</t>
-  </si>
-  <si>
-    <t>🩶 Grey</t>
-  </si>
-  <si>
-    <t>→ J1:14</t>
-  </si>
-  <si>
-    <t>MESA:TB6:6→</t>
-  </si>
-  <si>
-    <t>Y_MAX</t>
-  </si>
-  <si>
-    <t>→ J1:15</t>
-  </si>
-  <si>
-    <t>MESA:TB6:7→</t>
-  </si>
-  <si>
-    <t>Y1_HOME</t>
-  </si>
-  <si>
-    <t>→ J1:16</t>
-  </si>
-  <si>
-    <t>MESA:TB6:8→</t>
-  </si>
-  <si>
-    <t>Y2_HOME</t>
-  </si>
-  <si>
-    <t>→ J1:17</t>
-  </si>
-  <si>
-    <t>MESA:TB6:9→</t>
-  </si>
-  <si>
-    <t>X_MIN</t>
-  </si>
-  <si>
-    <t>→ J1:18</t>
-  </si>
-  <si>
-    <t>MESA:TB6:10→</t>
-  </si>
-  <si>
-    <t>X_MAX</t>
-  </si>
-  <si>
-    <t>→ J1:19</t>
-  </si>
-  <si>
-    <t>MESA:TB6:11→</t>
-  </si>
-  <si>
-    <t>X_HOME</t>
-  </si>
-  <si>
-    <t>→ J1:20</t>
-  </si>
-  <si>
-    <t>MESA:TB6:12→</t>
-  </si>
-  <si>
-    <t>Z_MIN</t>
-  </si>
-  <si>
-    <t>→ J1:21</t>
-  </si>
-  <si>
-    <t>MESA:TB6:13→</t>
-  </si>
-  <si>
-    <t>Z_MAX</t>
-  </si>
-  <si>
-    <t>13</t>
-  </si>
-  <si>
-    <t>→ J1:22</t>
-  </si>
-  <si>
-    <t>MESA:TB6:14→</t>
-  </si>
-  <si>
-    <t>Z_HOME</t>
-  </si>
-  <si>
-    <t>→ J1:23</t>
-  </si>
-  <si>
-    <t>MESA:TB6:15→</t>
-  </si>
-  <si>
-    <t>PROBE_IN</t>
-  </si>
-  <si>
-    <t>⬜️ White</t>
-  </si>
-  <si>
-    <t>→ FANS1:PWM</t>
-  </si>
-  <si>
-    <t>MESA:TB6:18→</t>
-  </si>
-  <si>
-    <t>FAN_PWM</t>
-  </si>
-  <si>
-    <t>PWM</t>
-  </si>
-  <si>
-    <t>→ J39:USB1</t>
-  </si>
-  <si>
-    <t>CPU1:USB1→</t>
-  </si>
-  <si>
-    <t>USB_HID</t>
-  </si>
-  <si>
-    <t>USB1</t>
-  </si>
-  <si>
-    <t>➖ not used</t>
-  </si>
-  <si>
-    <t>→ J38:USB1</t>
-  </si>
-  <si>
-    <t>CPU1:USB2→</t>
-  </si>
-  <si>
-    <t>USB_USER</t>
-  </si>
-  <si>
-    <t>USB2</t>
-  </si>
-  <si>
-    <t>Extend to monitor zone</t>
-  </si>
-  <si>
-    <t>→ J37:HDMI</t>
-  </si>
-  <si>
-    <t>CPU1:DP→</t>
-  </si>
-  <si>
-    <t>MONITOR</t>
-  </si>
-  <si>
-    <t>DP</t>
-  </si>
-  <si>
-    <t>Add in dp/hdmi adapter</t>
-  </si>
-  <si>
-    <t>→ RF1:1</t>
-  </si>
-  <si>
-    <t>CPU1:RF→</t>
-  </si>
-  <si>
-    <t>WIFI_EXT</t>
-  </si>
-  <si>
-    <t>RF</t>
-  </si>
-  <si>
-    <t>→ MESA:ETH</t>
-  </si>
-  <si>
-    <t>CPU1:ETH→</t>
-  </si>
-  <si>
-    <t>ETH_MESA</t>
-  </si>
-  <si>
-    <t>ETH</t>
-  </si>
-  <si>
-    <t>→ P11:8</t>
-  </si>
-  <si>
-    <t>P3:8→</t>
-  </si>
-  <si>
-    <t>→ P11:7</t>
-  </si>
-  <si>
-    <t>P3:7→</t>
-  </si>
-  <si>
-    <t>→ P11:6</t>
-  </si>
-  <si>
-    <t>P3:6→</t>
-  </si>
-  <si>
-    <t>→ P11:5</t>
-  </si>
-  <si>
-    <t>P3:5→</t>
-  </si>
-  <si>
-    <t>→ J18:1</t>
-  </si>
-  <si>
-    <t>J11:8→</t>
-  </si>
-  <si>
-    <t>→ J18:2</t>
-  </si>
-  <si>
-    <t>J11:7→</t>
-  </si>
-  <si>
-    <t>→ J18:3</t>
-  </si>
-  <si>
-    <t>J11:6→</t>
-  </si>
-  <si>
-    <t>→ J18:4</t>
-  </si>
-  <si>
-    <t>J11:5→</t>
-  </si>
-  <si>
-    <t>→ P30:8</t>
-  </si>
-  <si>
-    <t>P16:8→</t>
-  </si>
-  <si>
-    <t>→ P30:7</t>
-  </si>
-  <si>
-    <t>P16:7→</t>
-  </si>
-  <si>
-    <t>→ P30:6</t>
-  </si>
-  <si>
-    <t>P16:6→</t>
-  </si>
-  <si>
-    <t>→ P30:5</t>
-  </si>
-  <si>
-    <t>P16:5→</t>
-  </si>
-  <si>
-    <t>→ P11:4</t>
-  </si>
-  <si>
-    <t>P3:4→</t>
-  </si>
-  <si>
-    <t>→ P11:3</t>
-  </si>
-  <si>
-    <t>P3:3→</t>
-  </si>
-  <si>
-    <t>→ P11:2</t>
-  </si>
-  <si>
-    <t>P3:2→</t>
-  </si>
-  <si>
-    <t>→ P11:1</t>
-  </si>
-  <si>
-    <t>P3:1→</t>
-  </si>
-  <si>
-    <t>→ J16:4</t>
-  </si>
-  <si>
-    <t>J11:4→</t>
-  </si>
-  <si>
-    <t>→ J16:3</t>
-  </si>
-  <si>
-    <t>J11:3→</t>
-  </si>
-  <si>
-    <t>→ J16:2</t>
-  </si>
-  <si>
-    <t>J11:2→</t>
-  </si>
-  <si>
-    <t>→ J16:1</t>
-  </si>
-  <si>
-    <t>J11:1→</t>
-  </si>
-  <si>
-    <t>→ SM1</t>
-  </si>
-  <si>
-    <t>J30:8→</t>
-  </si>
-  <si>
-    <t>J30:7→</t>
-  </si>
-  <si>
-    <t>J30:6→</t>
-  </si>
-  <si>
-    <t>J30:5→</t>
-  </si>
-  <si>
-    <t>→ M1:1</t>
-  </si>
-  <si>
-    <t>VFD1:U→</t>
-  </si>
-  <si>
-    <t>SPINDLE_U</t>
-  </si>
-  <si>
-    <t>U</t>
-  </si>
-  <si>
     <t>→ M1:2</t>
   </si>
   <si>
@@ -3467,9 +3470,6 @@
   </si>
   <si>
     <t>TB4:3→</t>
-  </si>
-  <si>
-    <t>SPADE</t>
   </si>
   <si>
     <t>→ PS5:GND</t>
@@ -24703,7 +24703,7 @@
         <v>1</v>
       </c>
       <c r="N233" t="s" s="20">
-        <v>379</v>
+        <v>924</v>
       </c>
       <c r="O233" s="33">
         <v>10</v>
@@ -24736,14 +24736,14 @@
         <v>407</v>
       </c>
       <c r="F234" t="s" s="20">
-        <v>926</v>
+        <v>927</v>
       </c>
       <c r="G234" t="s" s="20">
         <v>296</v>
       </c>
       <c r="H234" s="20"/>
       <c r="I234" t="s" s="20">
-        <v>927</v>
+        <v>928</v>
       </c>
       <c r="J234" t="s" s="20">
         <v>329</v>
@@ -24756,7 +24756,7 @@
         <v>2</v>
       </c>
       <c r="N234" t="s" s="20">
-        <v>379</v>
+        <v>924</v>
       </c>
       <c r="O234" s="33">
         <v>10</v>
@@ -24789,14 +24789,14 @@
         <v>407</v>
       </c>
       <c r="F235" t="s" s="20">
-        <v>930</v>
+        <v>931</v>
       </c>
       <c r="G235" t="s" s="20">
         <v>296</v>
       </c>
       <c r="H235" s="20"/>
       <c r="I235" t="s" s="20">
-        <v>931</v>
+        <v>932</v>
       </c>
       <c r="J235" t="s" s="20">
         <v>329</v>
@@ -24809,7 +24809,7 @@
         <v>3</v>
       </c>
       <c r="N235" t="s" s="20">
-        <v>379</v>
+        <v>924</v>
       </c>
       <c r="O235" s="33">
         <v>10</v>
@@ -28355,7 +28355,7 @@
       </c>
       <c r="H302" s="20"/>
       <c r="I302" t="s" s="20">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="J302" t="s" s="20">
         <v>329</v>
@@ -28365,7 +28365,7 @@
       </c>
       <c r="L302" s="20"/>
       <c r="M302" t="s" s="20">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="N302" t="s" s="20">
         <v>329</v>
@@ -28914,7 +28914,7 @@
       </c>
       <c r="H313" s="20"/>
       <c r="I313" t="s" s="20">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="J313" t="s" s="20">
         <v>329</v>
@@ -28924,7 +28924,7 @@
       </c>
       <c r="L313" s="20"/>
       <c r="M313" t="s" s="20">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="N313" t="s" s="20">
         <v>329</v>
@@ -29279,7 +29279,7 @@
       </c>
       <c r="H320" s="20"/>
       <c r="I320" t="s" s="20">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="J320" t="s" s="20">
         <v>329</v>
@@ -29289,7 +29289,7 @@
       </c>
       <c r="L320" s="20"/>
       <c r="M320" t="s" s="20">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="N320" t="s" s="20">
         <v>329</v>
@@ -29585,7 +29585,7 @@
       </c>
       <c r="H326" s="20"/>
       <c r="I326" t="s" s="20">
-        <v>1066</v>
+        <v>1067</v>
       </c>
       <c r="J326" t="s" s="20">
         <v>329</v>
@@ -30096,20 +30096,20 @@
         <v>P0:PE→</v>
       </c>
       <c r="D336" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E336" t="s" s="19">
         <v>28</v>
       </c>
       <c r="F336" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G336" t="s" s="20">
         <v>153</v>
       </c>
       <c r="H336" s="20"/>
       <c r="I336" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="J336" t="s" s="20">
         <v>328</v>
@@ -30149,13 +30149,13 @@
         <v>TB1:2→</v>
       </c>
       <c r="D337" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E337" t="s" s="19">
         <v>28</v>
       </c>
       <c r="F337" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G337" t="s" s="20">
         <v>259</v>
@@ -30202,13 +30202,13 @@
         <v>TB4:3→</v>
       </c>
       <c r="D338" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E338" t="s" s="19">
         <v>28</v>
       </c>
       <c r="F338" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G338" t="s" s="20">
         <v>271</v>
@@ -30225,10 +30225,10 @@
       </c>
       <c r="L338" s="20"/>
       <c r="M338" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="N338" t="s" s="20">
-        <v>1132</v>
+        <v>379</v>
       </c>
       <c r="O338" s="33">
         <v>10</v>
@@ -30255,13 +30255,13 @@
         <v>TB4:18→</v>
       </c>
       <c r="D339" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E339" t="s" s="19">
         <v>28</v>
       </c>
       <c r="F339" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G339" t="s" s="20">
         <v>271</v>
@@ -30308,13 +30308,13 @@
         <v>TB4:16→</v>
       </c>
       <c r="D340" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E340" t="s" s="19">
         <v>28</v>
       </c>
       <c r="F340" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G340" t="s" s="20">
         <v>271</v>
@@ -30361,13 +30361,13 @@
         <v>TB4:14→</v>
       </c>
       <c r="D341" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E341" t="s" s="19">
         <v>28</v>
       </c>
       <c r="F341" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G341" t="s" s="20">
         <v>271</v>
@@ -30414,13 +30414,13 @@
         <v>TB4:12→</v>
       </c>
       <c r="D342" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E342" t="s" s="19">
         <v>28</v>
       </c>
       <c r="F342" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G342" t="s" s="20">
         <v>271</v>
@@ -30467,13 +30467,13 @@
         <v>TB4:10→</v>
       </c>
       <c r="D343" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E343" t="s" s="19">
         <v>28</v>
       </c>
       <c r="F343" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G343" t="s" s="20">
         <v>271</v>
@@ -30520,13 +30520,13 @@
         <v>TB4:8→</v>
       </c>
       <c r="D344" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E344" t="s" s="19">
         <v>28</v>
       </c>
       <c r="F344" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G344" t="s" s="20">
         <v>271</v>
@@ -30573,13 +30573,13 @@
         <v>TB4:6→</v>
       </c>
       <c r="D345" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E345" t="s" s="19">
         <v>28</v>
       </c>
       <c r="F345" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G345" t="s" s="20">
         <v>271</v>
@@ -30596,7 +30596,7 @@
       </c>
       <c r="L345" s="20"/>
       <c r="M345" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="N345" t="s" s="20">
         <v>328</v>
@@ -30626,13 +30626,13 @@
         <v>TB4:4→</v>
       </c>
       <c r="D346" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E346" t="s" s="19">
         <v>28</v>
       </c>
       <c r="F346" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G346" t="s" s="20">
         <v>271</v>
@@ -30649,10 +30649,10 @@
       </c>
       <c r="L346" s="20"/>
       <c r="M346" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="N346" t="s" s="20">
-        <v>379</v>
+        <v>924</v>
       </c>
       <c r="O346" s="33">
         <v>10</v>
@@ -30679,13 +30679,13 @@
         <v>TB4:20→</v>
       </c>
       <c r="D347" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E347" t="s" s="19">
         <v>28</v>
       </c>
       <c r="F347" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G347" t="s" s="20">
         <v>271</v>
@@ -30734,13 +30734,13 @@
         <v>TB4:2→</v>
       </c>
       <c r="D348" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E348" t="s" s="19">
         <v>28</v>
       </c>
       <c r="F348" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G348" t="s" s="20">
         <v>271</v>
@@ -30789,13 +30789,13 @@
         <v>P6:2→</v>
       </c>
       <c r="D349" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E349" t="s" s="19">
         <v>407</v>
       </c>
       <c r="F349" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G349" t="s" s="20">
         <v>188</v>
@@ -30815,7 +30815,7 @@
         <v>706</v>
       </c>
       <c r="N349" t="s" s="20">
-        <v>379</v>
+        <v>924</v>
       </c>
       <c r="O349" s="33">
         <v>10</v>
@@ -30842,13 +30842,13 @@
         <v>P6:1→</v>
       </c>
       <c r="D350" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E350" t="s" s="19">
         <v>407</v>
       </c>
       <c r="F350" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G350" t="s" s="20">
         <v>188</v>
@@ -30868,7 +30868,7 @@
         <v>4</v>
       </c>
       <c r="N350" t="s" s="20">
-        <v>379</v>
+        <v>924</v>
       </c>
       <c r="O350" s="33">
         <v>10</v>
@@ -30895,13 +30895,13 @@
         <v>P1:GND→</v>
       </c>
       <c r="D351" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E351" t="s" s="19">
         <v>407</v>
       </c>
       <c r="F351" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G351" t="s" s="20">
         <v>159</v>
@@ -30921,7 +30921,7 @@
         <v>706</v>
       </c>
       <c r="N351" t="s" s="20">
-        <v>379</v>
+        <v>924</v>
       </c>
       <c r="O351" s="33">
         <v>14</v>
@@ -30948,13 +30948,13 @@
         <v>J9:GND→</v>
       </c>
       <c r="D352" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E352" t="s" s="19">
         <v>407</v>
       </c>
       <c r="F352" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G352" t="s" s="20">
         <v>120</v>
@@ -30974,7 +30974,7 @@
         <v>706</v>
       </c>
       <c r="N352" t="s" s="20">
-        <v>379</v>
+        <v>924</v>
       </c>
       <c r="O352" s="33">
         <v>14</v>
@@ -31001,13 +31001,13 @@
         <v>P14:GND→</v>
       </c>
       <c r="D353" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E353" t="s" s="19">
         <v>407</v>
       </c>
       <c r="F353" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G353" t="s" s="20">
         <v>165</v>
@@ -31027,7 +31027,7 @@
         <v>706</v>
       </c>
       <c r="N353" t="s" s="20">
-        <v>379</v>
+        <v>924</v>
       </c>
       <c r="O353" s="33">
         <v>14</v>
@@ -31054,13 +31054,13 @@
         <v>J19:GND→</v>
       </c>
       <c r="D354" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E354" t="s" s="19">
         <v>407</v>
       </c>
       <c r="F354" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G354" t="s" s="20">
         <v>89</v>
@@ -31080,7 +31080,7 @@
         <v>9</v>
       </c>
       <c r="N354" t="s" s="20">
-        <v>379</v>
+        <v>924</v>
       </c>
       <c r="O354" s="33">
         <v>14</v>
@@ -31107,13 +31107,13 @@
         <v>P24:9→</v>
       </c>
       <c r="D355" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E355" t="s" s="19">
         <v>407</v>
       </c>
       <c r="F355" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G355" t="s" s="20">
         <v>174</v>
@@ -31133,7 +31133,7 @@
         <v>9</v>
       </c>
       <c r="N355" t="s" s="20">
-        <v>379</v>
+        <v>924</v>
       </c>
       <c r="O355" s="33">
         <v>14</v>
@@ -31160,20 +31160,20 @@
         <v>P35:PE→</v>
       </c>
       <c r="D356" t="s" s="21">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="E356" t="s" s="19">
         <v>407</v>
       </c>
       <c r="F356" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="G356" t="s" s="20">
         <v>181</v>
       </c>
       <c r="H356" s="20"/>
       <c r="I356" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="J356" t="s" s="20">
         <v>328</v>
@@ -31183,7 +31183,7 @@
       </c>
       <c r="L356" s="20"/>
       <c r="M356" t="s" s="20">
-        <v>1127</v>
+        <v>1128</v>
       </c>
       <c r="N356" t="s" s="20">
         <v>328</v>

</xml_diff>